<commit_message>
updated the files for testing the pipeline
</commit_message>
<xml_diff>
--- a/Task1/output/metrics_results/sales_analysis_report_metrics.xlsx
+++ b/Task1/output/metrics_results/sales_analysis_report_metrics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://zebra-my.sharepoint.com/personal/ak8963_zebra_com/Documents/Documents/Langextract_run/Task1/output/metrics_results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="11_2B59E82F90A953FA8181AB914B71807063DDC1F6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{545B851B-1582-456E-8006-59BF51499177}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="11_2B59E82F90A953FA8181AB914B71807063DDC1F6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12F76437-5FA8-4FF8-8051-C4A9966CD0AF}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -325,23 +325,23 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -359,6 +359,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -650,68 +654,69 @@
     <tabColor rgb="FF1F3864"/>
   </sheetPr>
   <dimension ref="A1:L25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.54296875" customWidth="1"/>
-    <col min="2" max="2" width="20.26953125" customWidth="1"/>
-    <col min="4" max="4" width="5.26953125" customWidth="1"/>
-    <col min="5" max="6" width="8.7265625" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="21.36328125" customWidth="1"/>
-    <col min="11" max="11" width="3.26953125" customWidth="1"/>
-    <col min="12" max="12" width="8.7265625" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="21.77734375" customWidth="1"/>
+    <col min="2" max="2" width="20.21875" customWidth="1"/>
+    <col min="4" max="4" width="9.88671875" customWidth="1"/>
+    <col min="5" max="5" width="6.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.77734375" customWidth="1"/>
+    <col min="7" max="7" width="21.33203125" customWidth="1"/>
+    <col min="11" max="11" width="3.21875" customWidth="1"/>
+    <col min="12" max="12" width="8.77734375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+    <row r="1" spans="1:12" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A2" s="15" t="s">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-    </row>
-    <row r="3" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+    </row>
+    <row r="3" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="13" t="s">
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-    </row>
-    <row r="4" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
+    </row>
+    <row r="4" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -733,7 +738,7 @@
       <c r="K4" s="10"/>
       <c r="L4" s="11"/>
     </row>
-    <row r="5" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -755,7 +760,7 @@
       <c r="K5" s="10"/>
       <c r="L5" s="11"/>
     </row>
-    <row r="6" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
@@ -777,7 +782,7 @@
       <c r="K6" s="10"/>
       <c r="L6" s="11"/>
     </row>
-    <row r="7" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
@@ -791,7 +796,7 @@
       <c r="G7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="16">
         <v>0</v>
       </c>
       <c r="I7" s="10"/>
@@ -799,7 +804,7 @@
       <c r="K7" s="10"/>
       <c r="L7" s="11"/>
     </row>
-    <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
@@ -813,7 +818,7 @@
       <c r="G8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="16">
         <v>0</v>
       </c>
       <c r="I8" s="10"/>
@@ -821,11 +826,11 @@
       <c r="K8" s="10"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="14">
         <v>28</v>
       </c>
       <c r="C9" s="10"/>
@@ -835,7 +840,7 @@
       <c r="G9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="16">
         <v>517.34</v>
       </c>
       <c r="I9" s="10"/>
@@ -843,7 +848,7 @@
       <c r="K9" s="10"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
@@ -857,7 +862,7 @@
       <c r="G10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H10" s="12">
+      <c r="H10" s="16">
         <v>517.34</v>
       </c>
       <c r="I10" s="10"/>
@@ -865,7 +870,7 @@
       <c r="K10" s="10"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
@@ -879,7 +884,7 @@
       <c r="G11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H11" s="17" t="s">
+      <c r="H11" s="15" t="s">
         <v>21</v>
       </c>
       <c r="I11" s="10"/>
@@ -887,7 +892,7 @@
       <c r="K11" s="10"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
@@ -905,7 +910,7 @@
       <c r="K12" s="10"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>23</v>
       </c>
@@ -923,7 +928,7 @@
       <c r="K13" s="10"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
@@ -941,7 +946,7 @@
       <c r="K14" s="10"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
@@ -959,7 +964,7 @@
       <c r="K15" s="10"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>26</v>
       </c>
@@ -977,11 +982,11 @@
       <c r="K16" s="10"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="14" t="s">
         <v>28</v>
       </c>
       <c r="C17" s="10"/>
@@ -995,23 +1000,23 @@
       <c r="K17" s="10"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="19" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="13" t="s">
+    <row r="19" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="14"/>
-      <c r="J19" s="14"/>
-      <c r="K19" s="14"/>
-      <c r="L19" s="14"/>
-    </row>
-    <row r="20" spans="1:12" ht="38.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13"/>
+      <c r="L19" s="13"/>
+    </row>
+    <row r="20" spans="1:12" ht="38.549999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>30</v>
       </c>
@@ -1034,7 +1039,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>1</v>
       </c>
@@ -1057,7 +1062,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>2</v>
       </c>
@@ -1080,7 +1085,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>3</v>
       </c>
@@ -1103,7 +1108,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>38</v>
       </c>
@@ -1133,10 +1138,17 @@
     <mergeCell ref="H14:L14"/>
     <mergeCell ref="H5:L5"/>
     <mergeCell ref="H8:L8"/>
-    <mergeCell ref="A19:L19"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="H16:L16"/>
-    <mergeCell ref="H13:L13"/>
+    <mergeCell ref="H7:L7"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="H6:L6"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="G3:L3"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="H4:L4"/>
+    <mergeCell ref="H9:L9"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="H12:L12"/>
     <mergeCell ref="B15:F15"/>
@@ -1145,22 +1157,15 @@
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="H17:L17"/>
     <mergeCell ref="H11:L11"/>
-    <mergeCell ref="H7:L7"/>
-    <mergeCell ref="A2:L2"/>
     <mergeCell ref="B12:F12"/>
-    <mergeCell ref="H6:L6"/>
     <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="B7:F7"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="H10:L10"/>
-    <mergeCell ref="G3:L3"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="H4:L4"/>
-    <mergeCell ref="H9:L9"/>
     <mergeCell ref="B14:F14"/>
+    <mergeCell ref="A19:L19"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="H16:L16"/>
+    <mergeCell ref="H13:L13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>